<commit_message>
temporarily hardcoded credentials because windows is windows
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smri_rpaops3\Documents\UiPath\RoboticEnterpriseFrameworkExcel\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53055FF2-6E1A-4DBF-8CF5-0470A0C6D2B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EADB53-86C7-4288-B7D0-853BDAACB4C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="0" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3130" yWindow="780" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -177,10 +177,10 @@
     <t>InputFilePath</t>
   </si>
   <si>
-    <t>Data\Input\UIDemo-Transactions.xlsx</t>
-  </si>
-  <si>
     <t>MaxTransactionThreshold</t>
+  </si>
+  <si>
+    <t>C:\Users\smri_rpaops3\Documents\UiPath\RoboticEnterpriseFrameworkExcel\Data\Input\UiDemo-Transactions.xlsx</t>
   </si>
 </sst>
 </file>
@@ -652,12 +652,12 @@
         <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B9">
         <v>10000</v>

</xml_diff>

<commit_message>
Reverted back to Initial Commit
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smri_rpaops3\Documents\UiPath\RoboticEnterpriseFrameworkExcel\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE09F2AB-066D-4CAD-8740-0AA343718F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53055FF2-6E1A-4DBF-8CF5-0470A0C6D2B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3130" yWindow="780" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4800" yWindow="0" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -177,10 +177,10 @@
     <t>InputFilePath</t>
   </si>
   <si>
+    <t>Data\Input\UIDemo-Transactions.xlsx</t>
+  </si>
+  <si>
     <t>MaxTransactionThreshold</t>
-  </si>
-  <si>
-    <t>C:\Users\smri_rpaops3\Documents\UiPath\RoboticEnterpriseFrameworkExcel\Data\Input\UiDemo-Transactions.xlsx</t>
   </si>
 </sst>
 </file>
@@ -652,12 +652,12 @@
         <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9">
         <v>10000</v>

</xml_diff>